<commit_message>
Ajuste no pprocesso automático de geração de rota fixa e melhoria na formatação a planilha de saída
</commit_message>
<xml_diff>
--- a/pdf/2026_03_06 PDF_operacao_2026_03_06 PDF_001_cl_oficial_programacao.xlsx
+++ b/pdf/2026_03_06 PDF_operacao_2026_03_06 PDF_001_cl_oficial_programacao.xlsx
@@ -120,15 +120,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -569,16 +576,16 @@
           <t>SERGIPE</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Data:</t>
         </is>
       </c>
-      <c r="H9" s="4" t="n"/>
+      <c r="H9" s="5" t="n"/>
       <c r="I9" s="2" t="n"/>
-      <c r="J9" s="5" t="n"/>
+      <c r="J9" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
@@ -587,11 +594,11 @@
         </is>
       </c>
       <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -617,1038 +624,1038 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>PROGRAMAÇÃO DE DISTRIBUIÇÃO DE PAX</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="8" t="n"/>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="8" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="9" t="n"/>
+      <c r="L13" s="9" t="n"/>
     </row>
     <row r="15" ht="57.75" customHeight="1">
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>EMBARCACAO</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>HR SAIDA ORIGEM</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>QUANT PAX EMBARQUE</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>ORIGEM</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>HORA CHEGADA DESTINO</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
         <is>
           <t>DESTINO</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>QUANT. PAX DESEMBARQUE</t>
         </is>
       </c>
-      <c r="I15" s="9" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>QUANT PAX A BORDO</t>
         </is>
       </c>
-      <c r="J15" s="9" t="inlineStr">
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>LINGADAS</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>OPERACAO DE TRANSBORDO</t>
         </is>
       </c>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="L15" s="10" t="inlineStr">
         <is>
           <t>OPERACAO</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>SURFER 1870</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>M9&gt;M6 = 13 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="12" t="n"/>
-      <c r="G16" s="12" t="n"/>
-      <c r="H16" s="12" t="n"/>
-      <c r="I16" s="12" t="n"/>
-      <c r="J16" s="12" t="n"/>
-      <c r="K16" s="12" t="n"/>
-      <c r="L16" s="12" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="13" t="n"/>
+      <c r="K16" s="13" t="n"/>
+      <c r="L16" s="13" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="13" t="inlineStr"/>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>05:10</t>
         </is>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="D17" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>05:14</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>M6</t>
         </is>
       </c>
-      <c r="H17" s="17" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>0(13)</t>
         </is>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="13" t="inlineStr"/>
-      <c r="K17" s="18" t="inlineStr">
+      <c r="J17" s="14" t="inlineStr"/>
+      <c r="K17" s="19" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="L17" s="13" t="inlineStr"/>
+      <c r="L17" s="14" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>SURFER 1931</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>TMIB&gt;M9&gt;TMIB = 48 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="12" t="n"/>
-      <c r="I19" s="12" t="n"/>
-      <c r="J19" s="12" t="n"/>
-      <c r="K19" s="12" t="n"/>
-      <c r="L19" s="12" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="13" t="inlineStr"/>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" s="14" t="inlineStr"/>
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="D20" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="F20" s="16" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>07:11</t>
         </is>
       </c>
-      <c r="G20" s="16" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="H20" s="17" t="inlineStr">
+      <c r="H20" s="18" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I20" s="18" t="n">
+      <c r="I20" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="J20" s="13" t="inlineStr"/>
-      <c r="K20" s="18" t="inlineStr">
+      <c r="J20" s="14" t="inlineStr"/>
+      <c r="K20" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L20" s="13" t="inlineStr">
+      <c r="L20" s="14" t="inlineStr">
         <is>
           <t>Em M9 pega 24 pax p/ TMIB</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="13" t="inlineStr"/>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr"/>
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>07:59</t>
         </is>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="D21" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="F21" s="16" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>08:40</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="H21" s="17" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>0(24)</t>
         </is>
       </c>
-      <c r="I21" s="18" t="n">
+      <c r="I21" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="13" t="inlineStr"/>
-      <c r="K21" s="18" t="inlineStr">
+      <c r="J21" s="14" t="inlineStr"/>
+      <c r="K21" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L21" s="13" t="inlineStr"/>
+      <c r="L21" s="14" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>SURFER 1930</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>TMIB&gt;M9&gt;TMIB = 28 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="12" t="n"/>
-      <c r="H23" s="12" t="n"/>
-      <c r="I23" s="12" t="n"/>
-      <c r="J23" s="12" t="n"/>
-      <c r="K23" s="12" t="n"/>
-      <c r="L23" s="12" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="13" t="inlineStr"/>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
+      <c r="K23" s="13" t="n"/>
+      <c r="L23" s="13" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="14" t="inlineStr"/>
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="D24" s="15" t="n">
+      <c r="D24" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="F24" s="16" t="inlineStr">
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>07:48</t>
         </is>
       </c>
-      <c r="G24" s="16" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="H24" s="17" t="inlineStr">
+      <c r="H24" s="18" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I24" s="18" t="n">
+      <c r="I24" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J24" s="13" t="inlineStr"/>
-      <c r="K24" s="18" t="inlineStr">
+      <c r="J24" s="14" t="inlineStr"/>
+      <c r="K24" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L24" s="13" t="inlineStr">
+      <c r="L24" s="14" t="inlineStr">
         <is>
           <t>Em M9 pega 4 pax p/ TMIB</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="13" t="inlineStr"/>
-      <c r="C25" s="16" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr"/>
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>08:16</t>
         </is>
       </c>
-      <c r="D25" s="15" t="n">
+      <c r="D25" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="F25" s="17" t="inlineStr">
         <is>
           <t>08:54</t>
         </is>
       </c>
-      <c r="G25" s="16" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="H25" s="18" t="inlineStr">
         <is>
           <t>0(4)</t>
         </is>
       </c>
-      <c r="I25" s="18" t="n">
+      <c r="I25" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="13" t="inlineStr"/>
-      <c r="K25" s="18" t="inlineStr">
+      <c r="J25" s="14" t="inlineStr"/>
+      <c r="K25" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L25" s="13" t="inlineStr"/>
+      <c r="L25" s="14" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>SURFER 1870</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>TMIB&gt;M9 = 24 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="12" t="n"/>
-      <c r="F27" s="12" t="n"/>
-      <c r="G27" s="12" t="n"/>
-      <c r="H27" s="12" t="n"/>
-      <c r="I27" s="12" t="n"/>
-      <c r="J27" s="12" t="n"/>
-      <c r="K27" s="12" t="n"/>
-      <c r="L27" s="12" t="n"/>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="13" t="n"/>
+      <c r="L27" s="13" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="B28" s="13" t="inlineStr"/>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr"/>
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>07:20</t>
         </is>
       </c>
-      <c r="D28" s="15" t="n">
+      <c r="D28" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F28" s="17" t="inlineStr">
         <is>
           <t>07:57</t>
         </is>
       </c>
-      <c r="G28" s="16" t="inlineStr">
+      <c r="G28" s="17" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="H28" s="17" t="inlineStr">
+      <c r="H28" s="18" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I28" s="18" t="n">
+      <c r="I28" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="13" t="inlineStr"/>
-      <c r="K28" s="18" t="inlineStr">
+      <c r="J28" s="14" t="inlineStr"/>
+      <c r="K28" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L28" s="13" t="inlineStr"/>
+      <c r="L28" s="14" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>SURFER 1931</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>TMIB&gt;M3&gt;M9&gt;M10 = 36 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="12" t="n"/>
-      <c r="I30" s="12" t="n"/>
-      <c r="J30" s="12" t="n"/>
-      <c r="K30" s="12" t="n"/>
-      <c r="L30" s="12" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="n"/>
+      <c r="J30" s="13" t="n"/>
+      <c r="K30" s="13" t="n"/>
+      <c r="L30" s="13" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="B31" s="13" t="inlineStr"/>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr"/>
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="D31" s="15" t="n">
+      <c r="D31" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="E31" s="13" t="inlineStr">
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>11:08</t>
         </is>
       </c>
-      <c r="G31" s="16" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="H31" s="17" t="inlineStr">
+      <c r="H31" s="18" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I31" s="18" t="n">
+      <c r="I31" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="J31" s="13" t="inlineStr"/>
-      <c r="K31" s="18" t="inlineStr">
+      <c r="J31" s="14" t="inlineStr"/>
+      <c r="K31" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L31" s="13" t="inlineStr"/>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="B32" s="13" t="inlineStr"/>
-      <c r="C32" s="16" t="inlineStr">
+      <c r="L31" s="14" t="inlineStr"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="B32" s="14" t="inlineStr"/>
+      <c r="C32" s="17" t="inlineStr">
         <is>
           <t>11:20</t>
         </is>
       </c>
-      <c r="D32" s="15" t="n">
+      <c r="D32" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="F32" s="17" t="inlineStr">
         <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="G32" s="16" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="H32" s="17" t="inlineStr">
+      <c r="H32" s="18" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="I32" s="18" t="n">
+      <c r="I32" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="J32" s="13" t="inlineStr"/>
-      <c r="K32" s="18" t="inlineStr">
+      <c r="J32" s="14" t="inlineStr"/>
+      <c r="K32" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L32" s="13" t="inlineStr">
+      <c r="L32" s="14" t="inlineStr">
         <is>
           <t>Em M9 pega 12 pax p/ M10</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="B33" s="13" t="inlineStr"/>
-      <c r="C33" s="16" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr"/>
+      <c r="C33" s="17" t="inlineStr">
         <is>
           <t>11:53</t>
         </is>
       </c>
-      <c r="D33" s="15" t="n">
+      <c r="D33" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="F33" s="16" t="inlineStr">
+      <c r="F33" s="17" t="inlineStr">
         <is>
           <t>11:56</t>
         </is>
       </c>
-      <c r="G33" s="16" t="inlineStr">
+      <c r="G33" s="17" t="inlineStr">
         <is>
           <t>M10</t>
         </is>
       </c>
-      <c r="H33" s="17" t="inlineStr">
+      <c r="H33" s="18" t="inlineStr">
         <is>
           <t>1(12)</t>
         </is>
       </c>
-      <c r="I33" s="18" t="n">
+      <c r="I33" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="13" t="inlineStr"/>
-      <c r="K33" s="18" t="inlineStr">
+      <c r="J33" s="14" t="inlineStr"/>
+      <c r="K33" s="19" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="L33" s="13" t="inlineStr"/>
+      <c r="L33" s="14" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>SURFER 1930</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>TMIB&gt;M9&gt;M5&gt;M1 = 24 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="12" t="n"/>
-      <c r="F35" s="12" t="n"/>
-      <c r="G35" s="12" t="n"/>
-      <c r="H35" s="12" t="n"/>
-      <c r="I35" s="12" t="n"/>
-      <c r="J35" s="12" t="n"/>
-      <c r="K35" s="12" t="n"/>
-      <c r="L35" s="12" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="n"/>
+      <c r="J35" s="13" t="n"/>
+      <c r="K35" s="13" t="n"/>
+      <c r="L35" s="13" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="B36" s="13" t="inlineStr"/>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr"/>
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>10:40</t>
         </is>
       </c>
-      <c r="D36" s="15" t="n">
+      <c r="D36" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="F36" s="16" t="inlineStr">
+      <c r="F36" s="17" t="inlineStr">
         <is>
           <t>11:18</t>
         </is>
       </c>
-      <c r="G36" s="16" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="H36" s="17" t="inlineStr">
+      <c r="H36" s="18" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="I36" s="18" t="n">
+      <c r="I36" s="19" t="n">
         <v>18</v>
       </c>
-      <c r="J36" s="13" t="inlineStr"/>
-      <c r="K36" s="18" t="inlineStr">
+      <c r="J36" s="14" t="inlineStr"/>
+      <c r="K36" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L36" s="13" t="inlineStr">
+      <c r="L36" s="14" t="inlineStr">
         <is>
           <t>Em M9 pega 4 pax p/ M1</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="B37" s="13" t="inlineStr"/>
-      <c r="C37" s="16" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr"/>
+      <c r="C37" s="17" t="inlineStr">
         <is>
           <t>11:28</t>
         </is>
       </c>
-      <c r="D37" s="15" t="n">
+      <c r="D37" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="E37" s="13" t="inlineStr">
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="F37" s="16" t="inlineStr">
+      <c r="F37" s="17" t="inlineStr">
         <is>
           <t>11:35</t>
         </is>
       </c>
-      <c r="G37" s="16" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
         <is>
           <t>M5</t>
         </is>
       </c>
-      <c r="H37" s="17" t="inlineStr">
+      <c r="H37" s="18" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I37" s="18" t="n">
+      <c r="I37" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="J37" s="13" t="inlineStr"/>
-      <c r="K37" s="18" t="inlineStr">
+      <c r="J37" s="14" t="inlineStr"/>
+      <c r="K37" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L37" s="13" t="inlineStr"/>
+      <c r="L37" s="14" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="B38" s="13" t="inlineStr"/>
-      <c r="C38" s="16" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr"/>
+      <c r="C38" s="17" t="inlineStr">
         <is>
           <t>11:38</t>
         </is>
       </c>
-      <c r="D38" s="15" t="n">
+      <c r="D38" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>M5</t>
         </is>
       </c>
-      <c r="F38" s="16" t="inlineStr">
+      <c r="F38" s="17" t="inlineStr">
         <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="G38" s="16" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="H38" s="17" t="inlineStr">
+      <c r="H38" s="18" t="inlineStr">
         <is>
           <t>11(4)</t>
         </is>
       </c>
-      <c r="I38" s="18" t="n">
+      <c r="I38" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="13" t="inlineStr"/>
-      <c r="K38" s="18" t="inlineStr">
+      <c r="J38" s="14" t="inlineStr"/>
+      <c r="K38" s="19" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="L38" s="13" t="inlineStr"/>
+      <c r="L38" s="14" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>SURFER 1870</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>TMIB&gt;M9&gt;M6&gt;B3&gt;B1 = 15 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="12" t="n"/>
-      <c r="G40" s="12" t="n"/>
-      <c r="H40" s="12" t="n"/>
-      <c r="I40" s="12" t="n"/>
-      <c r="J40" s="12" t="n"/>
-      <c r="K40" s="12" t="n"/>
-      <c r="L40" s="12" t="n"/>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="B41" s="13" t="inlineStr"/>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="D40" s="13" t="n"/>
+      <c r="E40" s="13" t="n"/>
+      <c r="F40" s="13" t="n"/>
+      <c r="G40" s="13" t="n"/>
+      <c r="H40" s="13" t="n"/>
+      <c r="I40" s="13" t="n"/>
+      <c r="J40" s="13" t="n"/>
+      <c r="K40" s="13" t="n"/>
+      <c r="L40" s="13" t="n"/>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="14" t="inlineStr"/>
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>10:50</t>
         </is>
       </c>
-      <c r="D41" s="15" t="n">
+      <c r="D41" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E41" s="14" t="inlineStr">
         <is>
           <t>TMIB</t>
         </is>
       </c>
-      <c r="F41" s="16" t="inlineStr">
+      <c r="F41" s="17" t="inlineStr">
         <is>
           <t>11:27</t>
         </is>
       </c>
-      <c r="G41" s="16" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="H41" s="17" t="inlineStr">
+      <c r="H41" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I41" s="18" t="n">
+      <c r="I41" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="J41" s="13" t="inlineStr"/>
-      <c r="K41" s="18" t="inlineStr">
+      <c r="J41" s="14" t="inlineStr"/>
+      <c r="K41" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L41" s="13" t="inlineStr">
+      <c r="L41" s="14" t="inlineStr">
         <is>
           <t>Em M9 pega 4 pax p/ B1 e 1 pax p/ B3</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="B42" s="13" t="inlineStr"/>
-      <c r="C42" s="16" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr"/>
+      <c r="C42" s="17" t="inlineStr">
         <is>
           <t>11:32</t>
         </is>
       </c>
-      <c r="D42" s="15" t="n">
+      <c r="D42" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E42" s="14" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="F42" s="16" t="inlineStr">
+      <c r="F42" s="17" t="inlineStr">
         <is>
           <t>11:36</t>
         </is>
       </c>
-      <c r="G42" s="16" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
         <is>
           <t>M6</t>
         </is>
       </c>
-      <c r="H42" s="17" t="inlineStr">
+      <c r="H42" s="18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I42" s="18" t="n">
+      <c r="I42" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="J42" s="13" t="inlineStr"/>
-      <c r="K42" s="18" t="inlineStr">
+      <c r="J42" s="14" t="inlineStr"/>
+      <c r="K42" s="19" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="L42" s="13" t="inlineStr"/>
+      <c r="L42" s="14" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="B43" s="13" t="inlineStr"/>
-      <c r="C43" s="16" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr"/>
+      <c r="C43" s="17" t="inlineStr">
         <is>
           <t>11:38</t>
         </is>
       </c>
-      <c r="D43" s="15" t="n">
+      <c r="D43" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="E43" s="13" t="inlineStr">
+      <c r="E43" s="14" t="inlineStr">
         <is>
           <t>M6</t>
         </is>
       </c>
-      <c r="F43" s="16" t="inlineStr">
+      <c r="F43" s="17" t="inlineStr">
         <is>
           <t>11:42</t>
         </is>
       </c>
-      <c r="G43" s="16" t="inlineStr">
+      <c r="G43" s="17" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="H43" s="17" t="inlineStr">
+      <c r="H43" s="18" t="inlineStr">
         <is>
           <t>4(1)</t>
         </is>
       </c>
-      <c r="I43" s="18" t="n">
+      <c r="I43" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J43" s="13" t="inlineStr"/>
-      <c r="K43" s="18" t="inlineStr">
+      <c r="J43" s="14" t="inlineStr"/>
+      <c r="K43" s="19" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="L43" s="13" t="inlineStr"/>
+      <c r="L43" s="14" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="B44" s="13" t="inlineStr"/>
-      <c r="C44" s="16" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr"/>
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>11:47</t>
         </is>
       </c>
-      <c r="D44" s="15" t="n">
+      <c r="D44" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="E44" s="14" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="F44" s="16" t="inlineStr">
+      <c r="F44" s="17" t="inlineStr">
         <is>
           <t>11:51</t>
         </is>
       </c>
-      <c r="G44" s="16" t="inlineStr">
+      <c r="G44" s="17" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="H44" s="17" t="inlineStr">
+      <c r="H44" s="18" t="inlineStr">
         <is>
           <t>4(4)</t>
         </is>
       </c>
-      <c r="I44" s="18" t="n">
+      <c r="I44" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J44" s="13" t="inlineStr"/>
-      <c r="K44" s="18" t="inlineStr">
+      <c r="J44" s="14" t="inlineStr"/>
+      <c r="K44" s="19" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="L44" s="13" t="inlineStr"/>
+      <c r="L44" s="14" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="B46" s="10" t="inlineStr">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>SURFER 1870</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>M9&gt;PGA3 = 7 PAX TRANSPORTADOS</t>
         </is>
       </c>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-      <c r="H46" s="12" t="n"/>
-      <c r="I46" s="12" t="n"/>
-      <c r="J46" s="12" t="n"/>
-      <c r="K46" s="12" t="n"/>
-      <c r="L46" s="12" t="n"/>
+      <c r="D46" s="13" t="n"/>
+      <c r="E46" s="13" t="n"/>
+      <c r="F46" s="13" t="n"/>
+      <c r="G46" s="13" t="n"/>
+      <c r="H46" s="13" t="n"/>
+      <c r="I46" s="13" t="n"/>
+      <c r="J46" s="13" t="n"/>
+      <c r="K46" s="13" t="n"/>
+      <c r="L46" s="13" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="B47" s="13" t="inlineStr"/>
-      <c r="C47" s="14" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr"/>
+      <c r="C47" s="15" t="inlineStr">
         <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="D47" s="15" t="n">
+      <c r="D47" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E47" s="14" t="inlineStr">
         <is>
           <t>M9</t>
         </is>
       </c>
-      <c r="F47" s="16" t="inlineStr">
+      <c r="F47" s="17" t="inlineStr">
         <is>
           <t>13:45</t>
         </is>
       </c>
-      <c r="G47" s="16" t="inlineStr">
+      <c r="G47" s="17" t="inlineStr">
         <is>
           <t>PGA3</t>
         </is>
       </c>
-      <c r="H47" s="17" t="inlineStr">
+      <c r="H47" s="18" t="inlineStr">
         <is>
           <t>0(7)</t>
         </is>
       </c>
-      <c r="I47" s="18" t="n">
+      <c r="I47" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J47" s="13" t="inlineStr"/>
-      <c r="K47" s="18" t="inlineStr">
+      <c r="J47" s="14" t="inlineStr"/>
+      <c r="K47" s="19" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="L47" s="13" t="inlineStr"/>
+      <c r="L47" s="14" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="B49" s="19" t="inlineStr">
+      <c r="B49" s="20" t="inlineStr">
         <is>
           <t>BARU TAURUS</t>
         </is>
       </c>
-      <c r="C49" s="20" t="n"/>
-      <c r="D49" s="20" t="n"/>
-      <c r="E49" s="20" t="n"/>
-      <c r="F49" s="20" t="n"/>
-      <c r="G49" s="20" t="n"/>
-      <c r="H49" s="20" t="n"/>
-      <c r="I49" s="20" t="n"/>
-      <c r="J49" s="20" t="n"/>
-      <c r="K49" s="20" t="n"/>
-      <c r="L49" s="20" t="n"/>
+      <c r="C49" s="21" t="n"/>
+      <c r="D49" s="21" t="n"/>
+      <c r="E49" s="21" t="n"/>
+      <c r="F49" s="21" t="n"/>
+      <c r="G49" s="21" t="n"/>
+      <c r="H49" s="21" t="n"/>
+      <c r="I49" s="21" t="n"/>
+      <c r="J49" s="21" t="n"/>
+      <c r="K49" s="21" t="n"/>
+      <c r="L49" s="21" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="B50" s="19" t="inlineStr">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>XOHÃ</t>
         </is>
       </c>
-      <c r="C50" s="20" t="n"/>
-      <c r="D50" s="20" t="n"/>
-      <c r="E50" s="20" t="n"/>
-      <c r="F50" s="20" t="n"/>
-      <c r="G50" s="20" t="n"/>
-      <c r="H50" s="20" t="n"/>
-      <c r="I50" s="20" t="n"/>
-      <c r="J50" s="20" t="n"/>
-      <c r="K50" s="20" t="n"/>
-      <c r="L50" s="20" t="n"/>
+      <c r="C50" s="21" t="n"/>
+      <c r="D50" s="21" t="n"/>
+      <c r="E50" s="21" t="n"/>
+      <c r="F50" s="21" t="n"/>
+      <c r="G50" s="21" t="n"/>
+      <c r="H50" s="21" t="n"/>
+      <c r="I50" s="21" t="n"/>
+      <c r="J50" s="21" t="n"/>
+      <c r="K50" s="21" t="n"/>
+      <c r="L50" s="21" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="21" t="inlineStr">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>OBSERVAÇÃO</t>
         </is>
       </c>
-      <c r="C52" s="8" t="n"/>
-      <c r="D52" s="8" t="n"/>
-      <c r="E52" s="8" t="n"/>
-      <c r="F52" s="8" t="n"/>
-      <c r="G52" s="8" t="n"/>
-      <c r="H52" s="8" t="n"/>
-      <c r="I52" s="8" t="n"/>
-      <c r="J52" s="8" t="n"/>
-      <c r="K52" s="8" t="n"/>
-      <c r="L52" s="8" t="n"/>
+      <c r="C52" s="9" t="n"/>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="F52" s="9" t="n"/>
+      <c r="G52" s="9" t="n"/>
+      <c r="H52" s="9" t="n"/>
+      <c r="I52" s="9" t="n"/>
+      <c r="J52" s="9" t="n"/>
+      <c r="K52" s="9" t="n"/>
+      <c r="L52" s="9" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>*Não iniciar a navegação com pax que não esteja no manifesto sem a autorização do CL</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>*Não coletar carga que não esteja no manifesto sem a autorização do CL;</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>*Essa programação pode sofrer alterações de horário, origem, destino, roteiro e embarcação.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="28.5" customHeight="1">
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>*Caso haja alguma outra demanda emergencial, deve ser enviado um e-mail pelo GIO da plataforma, para a célula do Planejamento PTMA2 (cc-ptma2-prog.transp.se-ba@petrobras.com.br) e para APMA9 (Controlador Logístico de PCM-09)</t>
         </is>

</xml_diff>